<commit_message>
Apply fact-check tweaks + pull two out-of-era photos from Unit 6
- US.50 chart: Midway data label now "≈362" (sources range 307–362).
- US.47 chart: "Germany & Austria" updated 210,000 → 225,000 (USHMM combined).
- Roster Photos tab: removed the two out-of-era photos (Unit 6 photo set
  now 40): US.57 interstate-highway (1956) and US.58 Truman/NATO (1949) —
  Cold War, not WWII. Files remain in Drive for re-tagging to the Cold War unit.
- Refreshed the US.47/US.50 analyst verdicts and FACTCHECK_REPORT.md action
  list to mark these as done. Open items remain: standardize the two Iwo Jima
  images on the LOC PD copy; confirm placement of five topic/standard mismatches.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VjU3H1SQFm1wNnvNkiXie5
</commit_message>
<xml_diff>
--- a/00_START_HERE/UNIT6_VISUAL_ASSETS/Unit6_Visual_QC_Roster.xlsx
+++ b/00_START_HERE/UNIT6_VISUAL_ASSETS/Unit6_Visual_QC_Roster.xlsx
@@ -1006,7 +1006,7 @@
       <c r="N10" s="4" t="inlineStr"/>
       <c r="O10" s="20" t="inlineStr">
         <is>
-          <t>VERIFIED (approx) — consistent w/ USHMM; ~6M total. Ger&amp;Austria 210k≈225k. Labeled estimates.</t>
+          <t>VERIFIED (approx) — consistent w/ USHMM; ~6M total. Ger&amp;Austria set to 225,000 (applied). Labeled estimates.</t>
         </is>
       </c>
       <c r="P10" s="4" t="inlineStr"/>
@@ -1110,7 +1110,7 @@
       <c r="N12" s="4" t="inlineStr"/>
       <c r="O12" s="20" t="inlineStr">
         <is>
-          <t>VERIFIED — D-Day 2,501; Iwo Jima 6,821; Okinawa 12,520. Midway ≈362 (range 307–362).</t>
+          <t>VERIFIED — D-Day 2,501; Iwo Jima 6,821; Okinawa 12,520; Midway ≈362 (label applied).</t>
         </is>
       </c>
       <c r="P12" s="4" t="inlineStr"/>
@@ -2261,7 +2261,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K47"/>
+  <dimension ref="A1:K45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -3856,17 +3856,17 @@
       </c>
       <c r="B44" s="16" t="inlineStr">
         <is>
-          <t>US.57</t>
+          <t>US.58</t>
         </is>
       </c>
       <c r="C44" s="17" t="inlineStr">
         <is>
-          <t>US.57_interstate_highway_1950s.jpg</t>
+          <t>US.58_cordell-hull-signing-un-charter.jpg</t>
         </is>
       </c>
       <c r="D44" s="27" t="inlineStr">
         <is>
-          <t>interstate_highway_1950s</t>
+          <t>cordell hull signing un charter</t>
         </is>
       </c>
       <c r="E44" s="19" t="inlineStr">
@@ -3879,9 +3879,9 @@
           <t>Cited (Drive) — prev. reviewed</t>
         </is>
       </c>
-      <c r="G44" s="28" t="inlineStr">
-        <is>
-          <t>OUT OF ERA: Interstate Highway (1956) is Cold War, not US.57 (Yalta/Potsdam). Remove from Unit 6 / re-tag.</t>
+      <c r="G44" s="20" t="inlineStr">
+        <is>
+          <t>VERIFIED: Hull, too ill for San Francisco, signed the Charter at the State Dept, Washington, Jul 1945. TN connection.</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr"/>
@@ -3900,12 +3900,12 @@
       </c>
       <c r="C45" s="17" t="inlineStr">
         <is>
-          <t>US.58_cordell-hull-signing-un-charter.jpg</t>
+          <t>US.58_declaration-by-united-nations-1942.jpg</t>
         </is>
       </c>
       <c r="D45" s="27" t="inlineStr">
         <is>
-          <t>cordell hull signing un charter</t>
+          <t>declaration by united nations 1942</t>
         </is>
       </c>
       <c r="E45" s="19" t="inlineStr">
@@ -3918,93 +3918,15 @@
           <t>Cited (Drive) — prev. reviewed</t>
         </is>
       </c>
-      <c r="G45" s="20" t="inlineStr">
-        <is>
-          <t>VERIFIED: Hull, too ill for San Francisco, signed the Charter at the State Dept, Washington, Jul 1945. TN connection.</t>
+      <c r="G45" s="21" t="inlineStr">
+        <is>
+          <t>Declaration by United Nations, Jan 1 1942. OK (UN origins).</t>
         </is>
       </c>
       <c r="H45" s="4" t="inlineStr"/>
       <c r="I45" s="4" t="inlineStr"/>
       <c r="J45" s="4" t="inlineStr"/>
       <c r="K45" s="4" t="inlineStr"/>
-    </row>
-    <row r="46" ht="30" customHeight="1">
-      <c r="A46" s="15" t="n">
-        <v>41</v>
-      </c>
-      <c r="B46" s="16" t="inlineStr">
-        <is>
-          <t>US.58</t>
-        </is>
-      </c>
-      <c r="C46" s="17" t="inlineStr">
-        <is>
-          <t>US.58_declaration-by-united-nations-1942.jpg</t>
-        </is>
-      </c>
-      <c r="D46" s="27" t="inlineStr">
-        <is>
-          <t>declaration by united nations 1942</t>
-        </is>
-      </c>
-      <c r="E46" s="19" t="inlineStr">
-        <is>
-          <t>View in Drive</t>
-        </is>
-      </c>
-      <c r="F46" s="27" t="inlineStr">
-        <is>
-          <t>Cited (Drive) — prev. reviewed</t>
-        </is>
-      </c>
-      <c r="G46" s="21" t="inlineStr">
-        <is>
-          <t>Declaration by United Nations, Jan 1 1942. OK (UN origins).</t>
-        </is>
-      </c>
-      <c r="H46" s="4" t="inlineStr"/>
-      <c r="I46" s="4" t="inlineStr"/>
-      <c r="J46" s="4" t="inlineStr"/>
-      <c r="K46" s="4" t="inlineStr"/>
-    </row>
-    <row r="47" ht="30" customHeight="1">
-      <c r="A47" s="15" t="n">
-        <v>42</v>
-      </c>
-      <c r="B47" s="16" t="inlineStr">
-        <is>
-          <t>US.58</t>
-        </is>
-      </c>
-      <c r="C47" s="17" t="inlineStr">
-        <is>
-          <t>US.58_truman_nato_signing_1949.jpg</t>
-        </is>
-      </c>
-      <c r="D47" s="27" t="inlineStr">
-        <is>
-          <t>truman_nato_signing_1949</t>
-        </is>
-      </c>
-      <c r="E47" s="19" t="inlineStr">
-        <is>
-          <t>View in Drive</t>
-        </is>
-      </c>
-      <c r="F47" s="27" t="inlineStr">
-        <is>
-          <t>Cited (Drive) — prev. reviewed</t>
-        </is>
-      </c>
-      <c r="G47" s="28" t="inlineStr">
-        <is>
-          <t>OUT OF ERA: NATO (1949) is Cold War, not UN founding US.58. Re-tag. (Drive lists image/gif despite .jpg — verify format.)</t>
-        </is>
-      </c>
-      <c r="H47" s="4" t="inlineStr"/>
-      <c r="I47" s="4" t="inlineStr"/>
-      <c r="J47" s="4" t="inlineStr"/>
-      <c r="K47" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -4015,7 +3937,7 @@
     <mergeCell ref="A1:K1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="H6:H47" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H6:H45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Accept,Needs fix,Reject,Re-tag,Remove"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4060,8 +3982,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId39"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId42"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Cite LOC for Iwo Jima photos + record photo re-tag decisions
- Iwo Jima flag-raising (US.49, US.51): switch citation to the Library of
  Congress public-domain copy (Rosenthal/AP 1945; loc.gov item 96515062,
  confirm LC call no.); same image — keep one.
- Re-tag the five topic/standard mismatches to their correct standard:
  women_welders→US.52, war_bonds→US.55, mochida→US.54 (poss. dup),
  tuskegee→US.51 (poss. dup), atomic_hiroshima→US.56 (fills gap).
- Roster Tab 3 fact-check notes and FACTCHECK_REPORT.md updated (B2/B3 +
  action list marked done).

Note: the Drive connector exposes copy/create only (no rename/delete), so
the actual Drive filename-prefix rename is a manual step; decisions are
recorded per-row in the roster.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VjU3H1SQFm1wNnvNkiXie5
</commit_message>
<xml_diff>
--- a/00_START_HERE/UNIT6_VISUAL_ASSETS/Unit6_Visual_QC_Roster.xlsx
+++ b/00_START_HERE/UNIT6_VISUAL_ASSETS/Unit6_Visual_QC_Roster.xlsx
@@ -185,7 +185,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -264,9 +264,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2826,9 +2823,9 @@
           <t>Cited (Drive) — prev. reviewed</t>
         </is>
       </c>
-      <c r="G17" s="28" t="inlineStr">
-        <is>
-          <t>PLACEMENT: home-front image under US.48 (Entry) — fits US.52/US.55.</t>
+      <c r="G17" s="21" t="inlineStr">
+        <is>
+          <t>RE-TAG -&gt; US.52 (Women in WWII): rename Drive prefix to US.52_. Home-front women workers.</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr"/>
@@ -2904,9 +2901,9 @@
           <t>Cited (Drive) — prev. reviewed</t>
         </is>
       </c>
-      <c r="G19" s="28" t="inlineStr">
-        <is>
-          <t>PLACEMENT: home-front poster under US.49 (Leaders) — fits US.55.</t>
+      <c r="G19" s="21" t="inlineStr">
+        <is>
+          <t>RE-TAG -&gt; US.55 (Home Front): rename Drive prefix to US.55_. War-bonds poster.</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr"/>
@@ -2945,7 +2942,7 @@
       </c>
       <c r="G20" s="21" t="inlineStr">
         <is>
-          <t>Rosenthal, Feb 23 1945. RIGHTS: widely PD (LOC/Wikimedia); AP asserted — use LOC copy. Topic fits US.50.</t>
+          <t>CITE LOC: Rosenthal (AP), Feb 23 1945 — use the Library of Congress Prints &amp; Photographs PUBLIC-DOMAIN copy (loc.gov item 96515062; confirm LC call no.). PD (copyright not renewed). Topic also fits US.50.</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr"/>
@@ -3062,7 +3059,7 @@
       </c>
       <c r="G23" s="21" t="inlineStr">
         <is>
-          <t>Lange 'Mochida family' Apr 1942. PLACEMENT: internment under US.50 (Battles) — fits US.54.</t>
+          <t>RE-TAG -&gt; US.54 (Internment): rename Drive prefix to US.54_. POSSIBLE DUPLICATE of US.54 Mochida-family photo — keep the better copy.</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr"/>
@@ -3179,7 +3176,7 @@
       </c>
       <c r="G26" s="21" t="inlineStr">
         <is>
-          <t>Rosenthal Iwo Jima. RIGHTS: widely PD; AP asserted — use LOC copy. Topic fits US.50.</t>
+          <t>CITE LOC: Rosenthal (AP), Feb 23 1945 — use the LOC Prints &amp; Photographs PD copy (loc.gov item 96515062; confirm LC call no.). Duplicate of the US.49 Iwo Jima — keep one. Topic fits US.50.</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr"/>
@@ -3216,9 +3213,9 @@
           <t>Cited (Drive) — prev. reviewed</t>
         </is>
       </c>
-      <c r="G27" s="28" t="inlineStr">
-        <is>
-          <t>PLACEMENT: Tuskegee under US.52 (Women) — fits US.51 (dup subject).</t>
+      <c r="G27" s="21" t="inlineStr">
+        <is>
+          <t>RE-TAG -&gt; US.51 (Special Forces): rename Drive prefix to US.51_. POSSIBLE DUPLICATE of US.51 Tuskegee photo — keep the better copy.</t>
         </is>
       </c>
       <c r="H27" s="4" t="inlineStr"/>
@@ -3372,9 +3369,9 @@
           <t>Cited (Drive) — prev. reviewed</t>
         </is>
       </c>
-      <c r="G31" s="28" t="inlineStr">
-        <is>
-          <t>PLACEMENT: atomic bomb under US.53 (African Americans) — fits US.56.</t>
+      <c r="G31" s="21" t="inlineStr">
+        <is>
+          <t>RE-TAG -&gt; US.56 (Manhattan Project): rename Drive prefix to US.56_. Fills the Hiroshima gap in US.56.</t>
         </is>
       </c>
       <c r="H31" s="4" t="inlineStr"/>

</xml_diff>